<commit_message>
chore: update baseline table (new column structure)
</commit_message>
<xml_diff>
--- a/钢铁指挥官兵种单位数据表7.29.xlsx
+++ b/钢铁指挥官兵种单位数据表7.29.xlsx
@@ -1,25 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr defaultThemeVersion="202300"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\Program\MechabellumData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C4544923-FCE4-4D8E-AD5A-28C88D1413E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{D1927B3C-EF77-46E7-A059-8E1E26F4DFE2}"/>
+    <workbookView windowWidth="21942" windowHeight="9805"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -31,15 +27,12 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="70">
   <si>
     <t>兵种名称</t>
   </si>
@@ -53,7 +46,16 @@
     <t>移速</t>
   </si>
   <si>
-    <t>单次攻击</t>
+    <t>攻击力</t>
+  </si>
+  <si>
+    <t>对单输出</t>
+  </si>
+  <si>
+    <t>爆发峰值</t>
+  </si>
+  <si>
+    <t>对单DPS</t>
   </si>
   <si>
     <t>溅射范围</t>
@@ -245,13 +247,20 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="6">
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="0_ "/>
+    <numFmt numFmtId="177" formatCode="0.00_ "/>
+  </numFmts>
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
-      <family val="2"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -260,14 +269,12 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Microsoft YaHei"/>
-      <family val="2"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="等线"/>
-      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -275,26 +282,161 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Microsoft YaHei"/>
-      <family val="2"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="等线"/>
-      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
       <name val="等线"/>
-      <family val="2"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="等线"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -325,8 +467,194 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -456,13 +784,255 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -493,6 +1063,9 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="176" fontId="3" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -517,18 +1090,65 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="177" fontId="3" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -577,7 +1197,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Display"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -610,26 +1230,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Narrow"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -662,23 +1265,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -840,21 +1426,19 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B13FD1B-1553-4445-9D2B-E5328139B2D0}">
-  <dimension ref="A1:S38"/>
-  <sheetFormatPr defaultRowHeight="14.15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:V38"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.1"/>
+  <cols>
+    <col min="8" max="8" width="11.6833333333333"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="29.15">
+    <row r="1" ht="29.15" spans="1:22">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -897,17 +1481,26 @@
       <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="4"/>
+      <c r="P1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="S1" s="4"/>
+      <c r="T1" s="4"/>
+      <c r="U1" s="4"/>
+      <c r="V1" s="4"/>
     </row>
-    <row r="2" spans="1:19">
+    <row r="2" spans="1:22">
       <c r="A2" s="5" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B2" s="6">
         <v>50</v>
@@ -934,31 +1527,40 @@
         <v>0</v>
       </c>
       <c r="J2" s="6">
+        <v>0</v>
+      </c>
+      <c r="K2" s="6">
+        <v>0</v>
+      </c>
+      <c r="L2" s="6">
+        <v>0</v>
+      </c>
+      <c r="M2" s="6">
         <v>5</v>
       </c>
-      <c r="K2" s="6">
+      <c r="N2" s="6">
         <v>6</v>
       </c>
-      <c r="L2" s="6">
-        <v>0</v>
-      </c>
-      <c r="M2" s="6">
-        <v>0</v>
-      </c>
-      <c r="N2" s="6">
-        <v>0</v>
-      </c>
-      <c r="O2" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="P2" s="4"/>
-      <c r="Q2" s="4"/>
-      <c r="R2" s="4"/>
+      <c r="O2" s="6">
+        <v>0</v>
+      </c>
+      <c r="P2" s="6">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="6">
+        <v>0</v>
+      </c>
+      <c r="R2" s="7" t="s">
+        <v>19</v>
+      </c>
       <c r="S2" s="4"/>
+      <c r="T2" s="4"/>
+      <c r="U2" s="4"/>
+      <c r="V2" s="4"/>
     </row>
-    <row r="3" spans="1:19">
+    <row r="3" spans="1:22">
       <c r="A3" s="8" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B3" s="9">
         <v>100</v>
@@ -973,43 +1575,54 @@
         <v>82</v>
       </c>
       <c r="F3" s="9">
+        <v>82</v>
+      </c>
+      <c r="G3" s="9">
+        <f>F3*M3</f>
+        <v>82</v>
+      </c>
+      <c r="H3" s="10">
+        <f>F3/J3</f>
+        <v>273.333333333333</v>
+      </c>
+      <c r="I3" s="9">
         <v>10</v>
       </c>
-      <c r="G3" s="9">
+      <c r="J3" s="9">
         <v>0.3</v>
       </c>
-      <c r="H3" s="9">
+      <c r="K3" s="9">
         <v>115</v>
       </c>
-      <c r="I3" s="9">
-        <v>0</v>
-      </c>
-      <c r="J3" s="9">
+      <c r="L3" s="9">
+        <v>0</v>
+      </c>
+      <c r="M3" s="9">
         <v>1</v>
       </c>
-      <c r="K3" s="9">
+      <c r="N3" s="9">
         <v>4</v>
       </c>
-      <c r="L3" s="9">
-        <v>0</v>
-      </c>
-      <c r="M3" s="9">
-        <v>0</v>
-      </c>
-      <c r="N3" s="9">
-        <v>0</v>
-      </c>
-      <c r="O3" s="10">
+      <c r="O3" s="9">
+        <v>0</v>
+      </c>
+      <c r="P3" s="9">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="9">
+        <v>0</v>
+      </c>
+      <c r="R3" s="11">
         <v>60</v>
       </c>
-      <c r="P3" s="4"/>
-      <c r="Q3" s="4"/>
-      <c r="R3" s="4"/>
       <c r="S3" s="4"/>
+      <c r="T3" s="4"/>
+      <c r="U3" s="4"/>
+      <c r="V3" s="4"/>
     </row>
-    <row r="4" spans="1:19">
+    <row r="4" spans="1:22">
       <c r="A4" s="8" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B4" s="9">
         <v>100</v>
@@ -1024,247 +1637,302 @@
         <v>365</v>
       </c>
       <c r="F4" s="9">
+        <v>365</v>
+      </c>
+      <c r="G4" s="9">
+        <f t="shared" ref="G4:G37" si="0">F4*M4</f>
+        <v>365</v>
+      </c>
+      <c r="H4" s="10">
+        <f t="shared" ref="H4:H37" si="1">F4/J4</f>
+        <v>405.555555555556</v>
+      </c>
+      <c r="I4" s="9">
         <v>7</v>
       </c>
-      <c r="G4" s="9">
+      <c r="J4" s="9">
         <v>0.9</v>
       </c>
-      <c r="H4" s="9">
+      <c r="K4" s="9">
         <v>95</v>
       </c>
-      <c r="I4" s="9">
+      <c r="L4" s="9">
         <v>0.5</v>
       </c>
-      <c r="J4" s="9">
+      <c r="M4" s="9">
         <v>1</v>
       </c>
-      <c r="K4" s="9">
+      <c r="N4" s="9">
         <v>4</v>
       </c>
-      <c r="L4" s="9">
-        <v>0</v>
-      </c>
-      <c r="M4" s="9">
+      <c r="O4" s="9">
+        <v>0</v>
+      </c>
+      <c r="P4" s="9">
         <v>100</v>
       </c>
-      <c r="N4" s="9">
+      <c r="Q4" s="9">
         <v>750</v>
       </c>
-      <c r="O4" s="11">
+      <c r="R4" s="12">
         <v>200</v>
       </c>
-      <c r="P4" s="4"/>
-      <c r="Q4" s="4"/>
-      <c r="R4" s="4"/>
       <c r="S4" s="4"/>
+      <c r="T4" s="4"/>
+      <c r="U4" s="4"/>
+      <c r="V4" s="4"/>
     </row>
-    <row r="5" spans="1:19">
+    <row r="5" spans="1:22">
       <c r="A5" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="12">
+        <v>22</v>
+      </c>
+      <c r="B5" s="13">
         <v>100</v>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="13">
         <v>879</v>
       </c>
-      <c r="D5" s="12">
+      <c r="D5" s="13">
         <v>10</v>
       </c>
-      <c r="E5" s="12">
+      <c r="E5" s="13">
         <v>246</v>
       </c>
-      <c r="F5" s="12">
+      <c r="F5" s="13">
+        <v>246</v>
+      </c>
+      <c r="G5" s="9">
+        <f t="shared" si="0"/>
+        <v>1230</v>
+      </c>
+      <c r="H5" s="10">
+        <f t="shared" si="1"/>
+        <v>102.5</v>
+      </c>
+      <c r="I5" s="13">
         <v>6</v>
       </c>
-      <c r="G5" s="12">
+      <c r="J5" s="13">
         <v>2.4</v>
       </c>
-      <c r="H5" s="12">
+      <c r="K5" s="13">
         <v>70</v>
       </c>
-      <c r="I5" s="12">
-        <v>0</v>
-      </c>
-      <c r="J5" s="12">
+      <c r="L5" s="13">
+        <v>0</v>
+      </c>
+      <c r="M5" s="13">
         <v>5</v>
       </c>
-      <c r="K5" s="12">
+      <c r="N5" s="13">
         <v>8</v>
       </c>
-      <c r="L5" s="12">
-        <v>0</v>
-      </c>
-      <c r="M5" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="N5" s="12">
+      <c r="O5" s="13">
+        <v>0</v>
+      </c>
+      <c r="P5" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q5" s="13">
         <v>750</v>
       </c>
-      <c r="O5" s="10">
+      <c r="R5" s="11">
         <v>200</v>
       </c>
-      <c r="P5" s="4"/>
-      <c r="Q5" s="4"/>
-      <c r="R5" s="4"/>
       <c r="S5" s="4"/>
+      <c r="T5" s="4"/>
+      <c r="U5" s="4"/>
+      <c r="V5" s="4"/>
     </row>
-    <row r="6" spans="1:19">
+    <row r="6" spans="1:22">
       <c r="A6" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" s="12">
+        <v>24</v>
+      </c>
+      <c r="B6" s="13">
         <v>100</v>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="13">
         <v>5028</v>
       </c>
-      <c r="D6" s="12">
-        <v>0</v>
-      </c>
-      <c r="E6" s="12">
+      <c r="D6" s="13">
+        <v>0</v>
+      </c>
+      <c r="E6" s="13">
         <v>2748</v>
       </c>
-      <c r="F6" s="12">
+      <c r="F6" s="13">
+        <v>2748</v>
+      </c>
+      <c r="G6" s="9">
+        <f t="shared" si="0"/>
+        <v>2748</v>
+      </c>
+      <c r="H6" s="10">
+        <f t="shared" si="1"/>
+        <v>1099.2</v>
+      </c>
+      <c r="I6" s="13">
         <v>5</v>
       </c>
-      <c r="G6" s="12">
+      <c r="J6" s="13">
         <v>2.5</v>
       </c>
-      <c r="H6" s="12">
+      <c r="K6" s="13">
         <v>125</v>
       </c>
-      <c r="I6" s="12">
-        <v>0</v>
-      </c>
-      <c r="J6" s="12">
+      <c r="L6" s="13">
+        <v>0</v>
+      </c>
+      <c r="M6" s="13">
         <v>1</v>
       </c>
-      <c r="K6" s="12">
+      <c r="N6" s="13">
         <v>4</v>
       </c>
-      <c r="L6" s="12">
-        <v>0</v>
-      </c>
-      <c r="M6" s="12">
-        <v>0</v>
-      </c>
-      <c r="N6" s="12">
-        <v>0</v>
-      </c>
-      <c r="O6" s="10">
+      <c r="O6" s="13">
+        <v>0</v>
+      </c>
+      <c r="P6" s="13">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="13">
+        <v>0</v>
+      </c>
+      <c r="R6" s="11">
         <v>60</v>
       </c>
-      <c r="P6" s="13"/>
-      <c r="Q6" s="13"/>
-      <c r="R6" s="13"/>
-      <c r="S6" s="13"/>
+      <c r="S6" s="14"/>
+      <c r="T6" s="14"/>
+      <c r="U6" s="14"/>
+      <c r="V6" s="14"/>
     </row>
-    <row r="7" spans="1:19">
+    <row r="7" spans="1:22">
       <c r="A7" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="12">
+        <v>25</v>
+      </c>
+      <c r="B7" s="13">
         <v>100</v>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="13">
         <v>1622</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="13">
         <v>8</v>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="13">
         <v>2329</v>
       </c>
-      <c r="F7" s="12">
-        <v>0</v>
-      </c>
-      <c r="G7" s="12">
+      <c r="F7" s="13">
+        <v>2329</v>
+      </c>
+      <c r="G7" s="9">
+        <f t="shared" si="0"/>
+        <v>2329</v>
+      </c>
+      <c r="H7" s="10">
+        <f t="shared" si="1"/>
+        <v>751.290322580645</v>
+      </c>
+      <c r="I7" s="13">
+        <v>0</v>
+      </c>
+      <c r="J7" s="13">
         <v>3.1</v>
       </c>
-      <c r="H7" s="12">
+      <c r="K7" s="13">
         <v>140</v>
       </c>
-      <c r="I7" s="12">
+      <c r="L7" s="13">
         <v>1</v>
       </c>
-      <c r="J7" s="12">
+      <c r="M7" s="13">
         <v>1</v>
       </c>
-      <c r="K7" s="12">
+      <c r="N7" s="13">
         <v>4</v>
       </c>
-      <c r="L7" s="12">
-        <v>0</v>
-      </c>
-      <c r="M7" s="12">
+      <c r="O7" s="13">
+        <v>0</v>
+      </c>
+      <c r="P7" s="13">
         <v>100</v>
       </c>
-      <c r="N7" s="12">
+      <c r="Q7" s="13">
         <v>650</v>
       </c>
-      <c r="O7" s="10">
+      <c r="R7" s="11">
         <v>200</v>
       </c>
-      <c r="P7" s="4"/>
-      <c r="Q7" s="4"/>
-      <c r="R7" s="4"/>
       <c r="S7" s="4"/>
+      <c r="T7" s="4"/>
+      <c r="U7" s="4"/>
+      <c r="V7" s="4"/>
     </row>
-    <row r="8" spans="1:19">
+    <row r="8" spans="1:22">
       <c r="A8" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="12">
+        <v>26</v>
+      </c>
+      <c r="B8" s="13">
         <v>100</v>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="13">
         <v>7425</v>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="13">
         <v>8</v>
       </c>
-      <c r="E8" s="12">
+      <c r="E8" s="13">
         <v>1309</v>
       </c>
-      <c r="F8" s="12">
-        <v>0</v>
-      </c>
-      <c r="G8" s="12">
+      <c r="F8" s="13">
+        <v>1309</v>
+      </c>
+      <c r="G8" s="9">
+        <f t="shared" si="0"/>
+        <v>1309</v>
+      </c>
+      <c r="H8" s="10">
+        <f t="shared" si="1"/>
+        <v>872.666666666667</v>
+      </c>
+      <c r="I8" s="13">
+        <v>0</v>
+      </c>
+      <c r="J8" s="13">
         <v>1.5</v>
       </c>
-      <c r="H8" s="12">
+      <c r="K8" s="13">
         <v>85</v>
       </c>
-      <c r="I8" s="12">
-        <v>0</v>
-      </c>
-      <c r="J8" s="12">
+      <c r="L8" s="13">
+        <v>0</v>
+      </c>
+      <c r="M8" s="13">
         <v>1</v>
       </c>
-      <c r="K8" s="12">
+      <c r="N8" s="13">
         <v>4</v>
       </c>
-      <c r="L8" s="12">
-        <v>0</v>
-      </c>
-      <c r="M8" s="12">
+      <c r="O8" s="13">
+        <v>0</v>
+      </c>
+      <c r="P8" s="13">
         <v>100</v>
       </c>
-      <c r="N8" s="12">
+      <c r="Q8" s="13">
         <v>750</v>
       </c>
-      <c r="O8" s="10">
+      <c r="R8" s="11">
         <v>200</v>
       </c>
-      <c r="P8" s="4"/>
-      <c r="Q8" s="4"/>
-      <c r="R8" s="4"/>
       <c r="S8" s="4"/>
+      <c r="T8" s="4"/>
+      <c r="U8" s="4"/>
+      <c r="V8" s="4"/>
     </row>
-    <row r="9" spans="1:19">
+    <row r="9" spans="1:22">
       <c r="A9" s="8" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B9" s="9">
         <v>100</v>
@@ -1279,94 +1947,116 @@
         <v>995</v>
       </c>
       <c r="F9" s="9">
-        <v>0</v>
+        <v>995</v>
       </c>
       <c r="G9" s="9">
+        <f t="shared" si="0"/>
+        <v>2985</v>
+      </c>
+      <c r="H9" s="10">
+        <f t="shared" si="1"/>
+        <v>301.515151515152</v>
+      </c>
+      <c r="I9" s="9">
+        <v>0</v>
+      </c>
+      <c r="J9" s="9">
         <v>3.3</v>
       </c>
-      <c r="H9" s="9">
+      <c r="K9" s="9">
         <v>100</v>
       </c>
-      <c r="I9" s="9">
+      <c r="L9" s="9">
         <v>0.5</v>
       </c>
-      <c r="J9" s="9">
+      <c r="M9" s="9">
         <v>3</v>
       </c>
-      <c r="K9" s="9">
+      <c r="N9" s="9">
         <v>8</v>
       </c>
-      <c r="L9" s="9">
-        <v>0</v>
-      </c>
-      <c r="M9" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="N9" s="9">
+      <c r="O9" s="9">
+        <v>0</v>
+      </c>
+      <c r="P9" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q9" s="9">
         <v>650</v>
       </c>
-      <c r="O9" s="11">
+      <c r="R9" s="12">
         <v>198</v>
       </c>
-      <c r="P9" s="4"/>
-      <c r="Q9" s="4"/>
-      <c r="R9" s="4"/>
       <c r="S9" s="4"/>
+      <c r="T9" s="4"/>
+      <c r="U9" s="4"/>
+      <c r="V9" s="4"/>
     </row>
-    <row r="10" spans="1:19">
+    <row r="10" spans="1:22">
       <c r="A10" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" s="12">
+        <v>29</v>
+      </c>
+      <c r="B10" s="13">
         <v>100</v>
       </c>
-      <c r="C10" s="12">
+      <c r="C10" s="13">
         <v>263</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="13">
         <v>16</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="13">
         <v>79</v>
       </c>
-      <c r="F10" s="12">
-        <v>0</v>
-      </c>
-      <c r="G10" s="12">
+      <c r="F10" s="13">
+        <v>79</v>
+      </c>
+      <c r="G10" s="9">
+        <f t="shared" si="0"/>
+        <v>1896</v>
+      </c>
+      <c r="H10" s="10">
+        <f t="shared" si="1"/>
+        <v>131.666666666667</v>
+      </c>
+      <c r="I10" s="13">
+        <v>0</v>
+      </c>
+      <c r="J10" s="13">
         <v>0.6</v>
       </c>
-      <c r="H10" s="12">
-        <v>0</v>
-      </c>
-      <c r="I10" s="12">
-        <v>0</v>
-      </c>
-      <c r="J10" s="12">
+      <c r="K10" s="13">
+        <v>0</v>
+      </c>
+      <c r="L10" s="13">
+        <v>0</v>
+      </c>
+      <c r="M10" s="13">
         <v>24</v>
       </c>
-      <c r="K10" s="12">
+      <c r="N10" s="13">
         <v>10</v>
       </c>
-      <c r="L10" s="12">
-        <v>0</v>
-      </c>
-      <c r="M10" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="N10" s="12">
+      <c r="O10" s="13">
+        <v>0</v>
+      </c>
+      <c r="P10" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q10" s="13">
         <v>450</v>
       </c>
-      <c r="O10" s="10">
+      <c r="R10" s="11">
         <v>192</v>
       </c>
-      <c r="P10" s="4"/>
-      <c r="Q10" s="4"/>
-      <c r="R10" s="4"/>
       <c r="S10" s="4"/>
+      <c r="T10" s="4"/>
+      <c r="U10" s="4"/>
+      <c r="V10" s="4"/>
     </row>
-    <row r="11" spans="1:19">
+    <row r="11" spans="1:22">
       <c r="A11" s="8" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B11" s="9">
         <v>100</v>
@@ -1381,94 +2071,116 @@
         <v>63</v>
       </c>
       <c r="F11" s="9">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="G11" s="9">
+        <f t="shared" si="0"/>
+        <v>1134</v>
+      </c>
+      <c r="H11" s="10">
+        <f t="shared" si="1"/>
+        <v>42</v>
+      </c>
+      <c r="I11" s="9">
+        <v>0</v>
+      </c>
+      <c r="J11" s="9">
         <v>1.5</v>
       </c>
-      <c r="H11" s="9">
+      <c r="K11" s="9">
         <v>75</v>
       </c>
-      <c r="I11" s="9">
+      <c r="L11" s="9">
         <v>1</v>
       </c>
-      <c r="J11" s="9">
+      <c r="M11" s="9">
         <v>18</v>
       </c>
-      <c r="K11" s="9">
+      <c r="N11" s="9">
         <v>10</v>
       </c>
-      <c r="L11" s="9">
-        <v>0</v>
-      </c>
-      <c r="M11" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="N11" s="9">
+      <c r="O11" s="9">
+        <v>0</v>
+      </c>
+      <c r="P11" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q11" s="9">
         <v>600</v>
       </c>
-      <c r="O11" s="11">
+      <c r="R11" s="12">
         <v>216</v>
       </c>
-      <c r="P11" s="4"/>
-      <c r="Q11" s="4"/>
-      <c r="R11" s="4"/>
       <c r="S11" s="4"/>
+      <c r="T11" s="4"/>
+      <c r="U11" s="4"/>
+      <c r="V11" s="4"/>
     </row>
-    <row r="12" spans="1:19">
+    <row r="12" spans="1:22">
       <c r="A12" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B12" s="12">
+        <v>33</v>
+      </c>
+      <c r="B12" s="13">
         <v>200</v>
       </c>
-      <c r="C12" s="12">
+      <c r="C12" s="13">
         <v>4222</v>
       </c>
-      <c r="D12" s="12">
+      <c r="D12" s="13">
         <v>9</v>
       </c>
-      <c r="E12" s="12">
+      <c r="E12" s="13">
         <v>27</v>
       </c>
-      <c r="F12" s="12">
+      <c r="F12" s="13">
+        <v>27</v>
+      </c>
+      <c r="G12" s="9">
+        <f t="shared" si="0"/>
+        <v>81</v>
+      </c>
+      <c r="H12" s="10">
+        <f t="shared" si="1"/>
+        <v>270</v>
+      </c>
+      <c r="I12" s="13">
         <v>7</v>
       </c>
-      <c r="G12" s="12">
+      <c r="J12" s="13">
         <v>0.1</v>
       </c>
-      <c r="H12" s="12">
+      <c r="K12" s="13">
         <v>75</v>
       </c>
-      <c r="I12" s="12">
-        <v>0</v>
-      </c>
-      <c r="J12" s="12">
+      <c r="L12" s="13">
+        <v>0</v>
+      </c>
+      <c r="M12" s="13">
         <v>3</v>
       </c>
-      <c r="K12" s="12">
+      <c r="N12" s="13">
         <v>10</v>
       </c>
-      <c r="L12" s="12">
-        <v>0</v>
-      </c>
-      <c r="M12" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="N12" s="12">
+      <c r="O12" s="13">
+        <v>0</v>
+      </c>
+      <c r="P12" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q12" s="13">
         <v>1400</v>
       </c>
-      <c r="O12" s="10">
+      <c r="R12" s="11">
         <v>402</v>
       </c>
-      <c r="P12" s="4"/>
-      <c r="Q12" s="4"/>
-      <c r="R12" s="4"/>
       <c r="S12" s="4"/>
+      <c r="T12" s="4"/>
+      <c r="U12" s="4"/>
+      <c r="V12" s="4"/>
     </row>
-    <row r="13" spans="1:19">
+    <row r="13" spans="1:22">
       <c r="A13" s="8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B13" s="9">
         <v>200</v>
@@ -1483,43 +2195,54 @@
         <v>3560</v>
       </c>
       <c r="F13" s="9">
+        <v>3560</v>
+      </c>
+      <c r="G13" s="9">
+        <f t="shared" si="0"/>
+        <v>3560</v>
+      </c>
+      <c r="H13" s="10">
+        <f t="shared" si="1"/>
+        <v>3955.55555555556</v>
+      </c>
+      <c r="I13" s="9">
         <v>6</v>
       </c>
-      <c r="G13" s="9">
+      <c r="J13" s="9">
         <v>0.9</v>
       </c>
-      <c r="H13" s="9">
-        <v>0</v>
-      </c>
-      <c r="I13" s="9">
-        <v>0</v>
-      </c>
-      <c r="J13" s="9">
+      <c r="K13" s="9">
+        <v>0</v>
+      </c>
+      <c r="L13" s="9">
+        <v>0</v>
+      </c>
+      <c r="M13" s="9">
         <v>1</v>
       </c>
-      <c r="K13" s="9">
+      <c r="N13" s="9">
         <v>9</v>
       </c>
-      <c r="L13" s="9">
+      <c r="O13" s="9">
         <v>50</v>
       </c>
-      <c r="M13" s="9">
+      <c r="P13" s="9">
         <v>200</v>
       </c>
-      <c r="N13" s="9">
+      <c r="Q13" s="9">
         <v>1150</v>
       </c>
-      <c r="O13" s="11">
+      <c r="R13" s="12">
         <v>400</v>
       </c>
-      <c r="P13" s="4"/>
-      <c r="Q13" s="4"/>
-      <c r="R13" s="4"/>
       <c r="S13" s="4"/>
+      <c r="T13" s="4"/>
+      <c r="U13" s="4"/>
+      <c r="V13" s="4"/>
     </row>
-    <row r="14" spans="1:19">
+    <row r="14" ht="13" customHeight="1" spans="1:22">
       <c r="A14" s="8" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B14" s="9">
         <v>200</v>
@@ -1531,97 +2254,120 @@
         <v>6</v>
       </c>
       <c r="E14" s="9">
+        <v>772</v>
+      </c>
+      <c r="F14" s="9">
+        <f>E14*4</f>
         <v>3088</v>
       </c>
-      <c r="F14" s="9">
+      <c r="G14" s="9">
+        <f t="shared" si="0"/>
+        <v>12352</v>
+      </c>
+      <c r="H14" s="10">
+        <f t="shared" si="1"/>
+        <v>467.878787878788</v>
+      </c>
+      <c r="I14" s="9">
         <v>5.5</v>
       </c>
-      <c r="G14" s="9">
+      <c r="J14" s="9">
         <v>6.6</v>
       </c>
-      <c r="H14" s="9">
+      <c r="K14" s="9">
         <v>180</v>
       </c>
-      <c r="I14" s="9">
-        <v>0</v>
-      </c>
-      <c r="J14" s="9">
+      <c r="L14" s="9">
+        <v>0</v>
+      </c>
+      <c r="M14" s="9">
         <v>4</v>
       </c>
-      <c r="K14" s="9">
+      <c r="N14" s="9">
         <v>10</v>
       </c>
-      <c r="L14" s="9">
+      <c r="O14" s="9">
         <v>50</v>
       </c>
-      <c r="M14" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="N14" s="9">
+      <c r="P14" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q14" s="9">
         <v>1100</v>
       </c>
-      <c r="O14" s="11">
+      <c r="R14" s="12">
         <v>400</v>
       </c>
-      <c r="P14" s="4"/>
-      <c r="Q14" s="4"/>
-      <c r="R14" s="4"/>
       <c r="S14" s="4"/>
+      <c r="T14" s="4"/>
+      <c r="U14" s="4"/>
+      <c r="V14" s="4"/>
     </row>
-    <row r="15" spans="1:19">
+    <row r="15" spans="1:22">
       <c r="A15" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="B15" s="12">
+        <v>38</v>
+      </c>
+      <c r="B15" s="13">
         <v>200</v>
       </c>
-      <c r="C15" s="12">
+      <c r="C15" s="13">
         <v>14886</v>
       </c>
-      <c r="D15" s="12">
+      <c r="D15" s="13">
         <v>8</v>
       </c>
-      <c r="E15" s="12">
+      <c r="E15" s="13">
         <v>6881</v>
       </c>
-      <c r="F15" s="12">
+      <c r="F15" s="13">
+        <v>6881</v>
+      </c>
+      <c r="G15" s="9">
+        <f t="shared" si="0"/>
+        <v>6881</v>
+      </c>
+      <c r="H15" s="10">
+        <f t="shared" si="1"/>
+        <v>2150.3125</v>
+      </c>
+      <c r="I15" s="13">
         <v>5</v>
       </c>
-      <c r="G15" s="12">
+      <c r="J15" s="13">
         <v>3.2</v>
       </c>
-      <c r="H15" s="12">
+      <c r="K15" s="13">
         <v>95</v>
       </c>
-      <c r="I15" s="12">
-        <v>0</v>
-      </c>
-      <c r="J15" s="12">
+      <c r="L15" s="13">
+        <v>0</v>
+      </c>
+      <c r="M15" s="13">
         <v>1</v>
       </c>
-      <c r="K15" s="12">
+      <c r="N15" s="13">
         <v>9</v>
       </c>
-      <c r="L15" s="12">
-        <v>0</v>
-      </c>
-      <c r="M15" s="12">
+      <c r="O15" s="13">
+        <v>0</v>
+      </c>
+      <c r="P15" s="13">
         <v>200</v>
       </c>
-      <c r="N15" s="12">
+      <c r="Q15" s="13">
         <v>1300</v>
       </c>
-      <c r="O15" s="10">
+      <c r="R15" s="11">
         <v>400</v>
       </c>
-      <c r="P15" s="4"/>
-      <c r="Q15" s="4"/>
-      <c r="R15" s="4"/>
       <c r="S15" s="4"/>
+      <c r="T15" s="4"/>
+      <c r="U15" s="4"/>
+      <c r="V15" s="4"/>
     </row>
-    <row r="16" spans="1:19">
+    <row r="16" spans="1:22">
       <c r="A16" s="8" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B16" s="9">
         <v>200</v>
@@ -1636,43 +2382,54 @@
         <v>608</v>
       </c>
       <c r="F16" s="9">
+        <v>608</v>
+      </c>
+      <c r="G16" s="9">
+        <f t="shared" si="0"/>
+        <v>3040</v>
+      </c>
+      <c r="H16" s="10">
+        <f t="shared" si="1"/>
+        <v>135.111111111111</v>
+      </c>
+      <c r="I16" s="9">
         <v>5</v>
       </c>
-      <c r="G16" s="9">
+      <c r="J16" s="9">
         <v>4.5</v>
       </c>
-      <c r="H16" s="9">
+      <c r="K16" s="9">
         <v>95</v>
       </c>
-      <c r="I16" s="9">
-        <v>0</v>
-      </c>
-      <c r="J16" s="9">
+      <c r="L16" s="9">
+        <v>0</v>
+      </c>
+      <c r="M16" s="9">
         <v>5</v>
       </c>
-      <c r="K16" s="9">
+      <c r="N16" s="9">
         <v>10</v>
       </c>
-      <c r="L16" s="9">
-        <v>0</v>
-      </c>
-      <c r="M16" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="N16" s="9">
+      <c r="O16" s="9">
+        <v>0</v>
+      </c>
+      <c r="P16" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q16" s="9">
         <v>1300</v>
       </c>
-      <c r="O16" s="11">
+      <c r="R16" s="12">
         <v>400</v>
       </c>
-      <c r="P16" s="4"/>
-      <c r="Q16" s="4"/>
-      <c r="R16" s="4"/>
       <c r="S16" s="4"/>
+      <c r="T16" s="4"/>
+      <c r="U16" s="4"/>
+      <c r="V16" s="4"/>
     </row>
-    <row r="17" spans="1:19">
+    <row r="17" spans="1:22">
       <c r="A17" s="8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B17" s="9">
         <v>200</v>
@@ -1687,43 +2444,54 @@
         <v>496</v>
       </c>
       <c r="F17" s="9">
+        <v>496</v>
+      </c>
+      <c r="G17" s="9">
+        <f t="shared" si="0"/>
+        <v>496</v>
+      </c>
+      <c r="H17" s="10">
+        <f t="shared" si="1"/>
+        <v>826.666666666667</v>
+      </c>
+      <c r="I17" s="9">
         <v>5</v>
       </c>
-      <c r="G17" s="9">
+      <c r="J17" s="9">
         <v>0.6</v>
       </c>
-      <c r="H17" s="9">
+      <c r="K17" s="9">
         <v>80</v>
       </c>
-      <c r="I17" s="9">
+      <c r="L17" s="9">
         <v>0.5</v>
       </c>
-      <c r="J17" s="9">
+      <c r="M17" s="9">
         <v>1</v>
       </c>
-      <c r="K17" s="9">
+      <c r="N17" s="9">
         <v>9</v>
       </c>
-      <c r="L17" s="9">
-        <v>0</v>
-      </c>
-      <c r="M17" s="9">
+      <c r="O17" s="9">
+        <v>0</v>
+      </c>
+      <c r="P17" s="9">
         <v>200</v>
       </c>
-      <c r="N17" s="9">
+      <c r="Q17" s="9">
         <v>1500</v>
       </c>
-      <c r="O17" s="11">
+      <c r="R17" s="12">
         <v>400</v>
       </c>
-      <c r="P17" s="4"/>
-      <c r="Q17" s="4"/>
-      <c r="R17" s="4"/>
       <c r="S17" s="4"/>
+      <c r="T17" s="4"/>
+      <c r="U17" s="4"/>
+      <c r="V17" s="4"/>
     </row>
-    <row r="18" spans="1:19">
+    <row r="18" spans="1:22">
       <c r="A18" s="8" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B18" s="9">
         <v>200</v>
@@ -1735,46 +2503,58 @@
         <v>16</v>
       </c>
       <c r="E18" s="9">
+        <v>1087</v>
+      </c>
+      <c r="F18" s="9">
+        <f>E18*2</f>
         <v>2174</v>
       </c>
-      <c r="F18" s="9">
+      <c r="G18" s="9">
+        <f t="shared" si="0"/>
+        <v>6522</v>
+      </c>
+      <c r="H18" s="10">
+        <f t="shared" si="1"/>
+        <v>724.666666666667</v>
+      </c>
+      <c r="I18" s="9">
         <v>3</v>
-      </c>
-      <c r="G18" s="9">
-        <v>3</v>
-      </c>
-      <c r="H18" s="9">
-        <v>65</v>
-      </c>
-      <c r="I18" s="9">
-        <v>1</v>
       </c>
       <c r="J18" s="9">
         <v>3</v>
       </c>
       <c r="K18" s="9">
+        <v>65</v>
+      </c>
+      <c r="L18" s="9">
+        <v>1</v>
+      </c>
+      <c r="M18" s="9">
+        <v>3</v>
+      </c>
+      <c r="N18" s="9">
         <v>10</v>
       </c>
-      <c r="L18" s="9">
+      <c r="O18" s="9">
         <v>50</v>
       </c>
-      <c r="M18" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="N18" s="9">
+      <c r="P18" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q18" s="9">
         <v>1000</v>
       </c>
-      <c r="O18" s="11">
+      <c r="R18" s="12">
         <v>408</v>
       </c>
-      <c r="P18" s="4"/>
-      <c r="Q18" s="4"/>
-      <c r="R18" s="4"/>
       <c r="S18" s="4"/>
+      <c r="T18" s="4"/>
+      <c r="U18" s="4"/>
+      <c r="V18" s="4"/>
     </row>
-    <row r="19" spans="1:19">
+    <row r="19" spans="1:22">
       <c r="A19" s="8" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B19" s="9">
         <v>200</v>
@@ -1789,298 +2569,364 @@
         <v>2814</v>
       </c>
       <c r="F19" s="9">
-        <v>0</v>
+        <v>2814</v>
       </c>
       <c r="G19" s="9">
+        <f t="shared" si="0"/>
+        <v>5628</v>
+      </c>
+      <c r="H19" s="10">
+        <f t="shared" si="1"/>
+        <v>827.647058823529</v>
+      </c>
+      <c r="I19" s="9">
+        <v>0</v>
+      </c>
+      <c r="J19" s="9">
         <v>3.4</v>
       </c>
-      <c r="H19" s="9">
+      <c r="K19" s="9">
         <v>120</v>
       </c>
-      <c r="I19" s="9">
+      <c r="L19" s="9">
         <v>1</v>
       </c>
-      <c r="J19" s="9">
+      <c r="M19" s="9">
         <v>2</v>
       </c>
-      <c r="K19" s="9">
+      <c r="N19" s="9">
         <v>8</v>
       </c>
-      <c r="L19" s="9">
+      <c r="O19" s="9">
         <v>50</v>
       </c>
-      <c r="M19" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="N19" s="9">
+      <c r="P19" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q19" s="9">
         <v>1300</v>
       </c>
-      <c r="O19" s="11">
+      <c r="R19" s="12">
         <v>400</v>
       </c>
-      <c r="P19" s="4"/>
-      <c r="Q19" s="4"/>
-      <c r="R19" s="4"/>
       <c r="S19" s="4"/>
+      <c r="T19" s="4"/>
+      <c r="U19" s="4"/>
+      <c r="V19" s="4"/>
     </row>
-    <row r="20" spans="1:19">
+    <row r="20" spans="1:22">
       <c r="A20" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="B20" s="12">
+        <v>45</v>
+      </c>
+      <c r="B20" s="13">
         <v>200</v>
       </c>
-      <c r="C20" s="12">
+      <c r="C20" s="13">
         <v>4571</v>
       </c>
-      <c r="D20" s="12">
+      <c r="D20" s="13">
         <v>16</v>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="13">
         <v>2605</v>
       </c>
-      <c r="F20" s="12">
-        <v>0</v>
-      </c>
-      <c r="G20" s="12">
+      <c r="F20" s="13">
+        <v>2605</v>
+      </c>
+      <c r="G20" s="9">
+        <f t="shared" si="0"/>
+        <v>10420</v>
+      </c>
+      <c r="H20" s="10">
+        <f t="shared" si="1"/>
+        <v>13025</v>
+      </c>
+      <c r="I20" s="13">
+        <v>0</v>
+      </c>
+      <c r="J20" s="13">
         <v>0.2</v>
       </c>
-      <c r="H20" s="12">
+      <c r="K20" s="13">
         <v>45</v>
       </c>
-      <c r="I20" s="12">
-        <v>0</v>
-      </c>
-      <c r="J20" s="12">
+      <c r="L20" s="13">
+        <v>0</v>
+      </c>
+      <c r="M20" s="13">
         <v>4</v>
       </c>
-      <c r="K20" s="12">
+      <c r="N20" s="13">
         <v>10</v>
       </c>
-      <c r="L20" s="12">
-        <v>0</v>
-      </c>
-      <c r="M20" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="N20" s="12">
+      <c r="O20" s="13">
+        <v>0</v>
+      </c>
+      <c r="P20" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q20" s="13">
         <v>1000</v>
       </c>
-      <c r="O20" s="10">
+      <c r="R20" s="11">
         <v>400</v>
       </c>
-      <c r="P20" s="4"/>
-      <c r="Q20" s="4"/>
-      <c r="R20" s="4"/>
       <c r="S20" s="4"/>
+      <c r="T20" s="4"/>
+      <c r="U20" s="4"/>
+      <c r="V20" s="4"/>
     </row>
-    <row r="21" spans="1:19">
+    <row r="21" spans="1:22">
       <c r="A21" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="B21" s="12">
+        <v>46</v>
+      </c>
+      <c r="B21" s="13">
         <v>200</v>
       </c>
-      <c r="C21" s="12">
+      <c r="C21" s="13">
         <v>3249</v>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="13">
         <v>8</v>
       </c>
-      <c r="E21" s="12">
+      <c r="E21" s="13">
         <v>600</v>
       </c>
-      <c r="F21" s="12">
-        <v>0</v>
-      </c>
-      <c r="G21" s="12">
+      <c r="F21" s="13">
+        <v>600</v>
+      </c>
+      <c r="G21" s="9">
+        <f t="shared" si="0"/>
+        <v>600</v>
+      </c>
+      <c r="H21" s="10">
+        <f t="shared" si="1"/>
+        <v>2000</v>
+      </c>
+      <c r="I21" s="13">
+        <v>0</v>
+      </c>
+      <c r="J21" s="13">
         <v>0.3</v>
       </c>
-      <c r="H21" s="12">
+      <c r="K21" s="13">
         <v>110</v>
       </c>
-      <c r="I21" s="12">
-        <v>0</v>
-      </c>
-      <c r="J21" s="12">
+      <c r="L21" s="13">
+        <v>0</v>
+      </c>
+      <c r="M21" s="13">
         <v>1</v>
       </c>
-      <c r="K21" s="12">
+      <c r="N21" s="13">
         <v>9</v>
       </c>
-      <c r="L21" s="12">
+      <c r="O21" s="13">
         <v>100</v>
       </c>
-      <c r="M21" s="12">
+      <c r="P21" s="13">
         <v>200</v>
       </c>
-      <c r="N21" s="12">
+      <c r="Q21" s="13">
         <v>560</v>
       </c>
-      <c r="O21" s="10">
+      <c r="R21" s="11">
         <v>400</v>
       </c>
-      <c r="P21" s="4"/>
-      <c r="Q21" s="4"/>
-      <c r="R21" s="4"/>
       <c r="S21" s="4"/>
+      <c r="T21" s="4"/>
+      <c r="U21" s="4"/>
+      <c r="V21" s="4"/>
     </row>
-    <row r="22" spans="1:19">
+    <row r="22" spans="1:22">
       <c r="A22" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="B22" s="12">
+        <v>47</v>
+      </c>
+      <c r="B22" s="13">
         <v>200</v>
       </c>
-      <c r="C22" s="12">
+      <c r="C22" s="13">
         <v>311</v>
       </c>
-      <c r="D22" s="12">
+      <c r="D22" s="13">
         <v>16</v>
       </c>
-      <c r="E22" s="12">
+      <c r="E22" s="13">
         <v>202</v>
       </c>
-      <c r="F22" s="12">
-        <v>0</v>
-      </c>
-      <c r="G22" s="12">
+      <c r="F22" s="13">
+        <v>202</v>
+      </c>
+      <c r="G22" s="9">
+        <f t="shared" si="0"/>
+        <v>2424</v>
+      </c>
+      <c r="H22" s="10">
+        <f t="shared" si="1"/>
+        <v>144.285714285714</v>
+      </c>
+      <c r="I22" s="13">
+        <v>0</v>
+      </c>
+      <c r="J22" s="13">
         <v>1.4</v>
       </c>
-      <c r="H22" s="12">
+      <c r="K22" s="13">
         <v>50</v>
       </c>
-      <c r="I22" s="12">
+      <c r="L22" s="13">
         <v>1</v>
       </c>
-      <c r="J22" s="12">
+      <c r="M22" s="13">
         <v>12</v>
       </c>
-      <c r="K22" s="12">
+      <c r="N22" s="13">
         <v>10</v>
       </c>
-      <c r="L22" s="12">
+      <c r="O22" s="13">
         <v>50</v>
       </c>
-      <c r="M22" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="N22" s="12">
+      <c r="P22" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q22" s="13">
         <v>900</v>
       </c>
-      <c r="O22" s="10">
+      <c r="R22" s="11">
         <v>408</v>
       </c>
-      <c r="P22" s="4"/>
-      <c r="Q22" s="4"/>
-      <c r="R22" s="4"/>
       <c r="S22" s="4"/>
+      <c r="T22" s="4"/>
+      <c r="U22" s="4"/>
+      <c r="V22" s="4"/>
     </row>
-    <row r="23" spans="1:19">
+    <row r="23" spans="1:22">
       <c r="A23" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="B23" s="12">
+        <v>49</v>
+      </c>
+      <c r="B23" s="13">
         <v>200</v>
       </c>
-      <c r="C23" s="12">
+      <c r="C23" s="13">
         <v>343</v>
       </c>
-      <c r="D23" s="12">
+      <c r="D23" s="13">
         <v>16</v>
       </c>
-      <c r="E23" s="12">
+      <c r="E23" s="13">
         <v>36</v>
       </c>
-      <c r="F23" s="12">
-        <v>0</v>
-      </c>
-      <c r="G23" s="12">
+      <c r="F23" s="13">
+        <v>36</v>
+      </c>
+      <c r="G23" s="9">
+        <f t="shared" si="0"/>
+        <v>432</v>
+      </c>
+      <c r="H23" s="10">
+        <f t="shared" si="1"/>
+        <v>90</v>
+      </c>
+      <c r="I23" s="13">
+        <v>0</v>
+      </c>
+      <c r="J23" s="13">
         <v>0.4</v>
       </c>
-      <c r="H23" s="12">
+      <c r="K23" s="13">
         <v>95</v>
       </c>
-      <c r="I23" s="12">
+      <c r="L23" s="13">
         <v>1</v>
       </c>
-      <c r="J23" s="12">
+      <c r="M23" s="13">
         <v>12</v>
       </c>
-      <c r="K23" s="12">
+      <c r="N23" s="13">
         <v>10</v>
       </c>
-      <c r="L23" s="12">
-        <v>0</v>
-      </c>
-      <c r="M23" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="N23" s="12">
+      <c r="O23" s="13">
+        <v>0</v>
+      </c>
+      <c r="P23" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q23" s="13">
         <v>1200</v>
       </c>
-      <c r="O23" s="10">
+      <c r="R23" s="11">
         <v>408</v>
       </c>
-      <c r="P23" s="4"/>
-      <c r="Q23" s="4"/>
-      <c r="R23" s="4"/>
       <c r="S23" s="4"/>
+      <c r="T23" s="4"/>
+      <c r="U23" s="4"/>
+      <c r="V23" s="4"/>
     </row>
-    <row r="24" spans="1:19">
+    <row r="24" spans="1:22">
       <c r="A24" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="B24" s="12">
+        <v>50</v>
+      </c>
+      <c r="B24" s="13">
         <v>300</v>
       </c>
-      <c r="C24" s="12">
+      <c r="C24" s="13">
         <v>18632</v>
       </c>
-      <c r="D24" s="12">
+      <c r="D24" s="13">
         <v>7</v>
       </c>
-      <c r="E24" s="12">
+      <c r="E24" s="13">
         <v>10650</v>
       </c>
-      <c r="F24" s="12">
+      <c r="F24" s="13">
+        <v>10650</v>
+      </c>
+      <c r="G24" s="9">
+        <f t="shared" si="0"/>
+        <v>10650</v>
+      </c>
+      <c r="H24" s="10">
+        <f t="shared" si="1"/>
+        <v>2366.66666666667</v>
+      </c>
+      <c r="I24" s="13">
         <v>15</v>
       </c>
-      <c r="G24" s="12">
+      <c r="J24" s="13">
         <v>4.5</v>
       </c>
-      <c r="H24" s="12">
+      <c r="K24" s="13">
         <v>100</v>
       </c>
-      <c r="I24" s="12">
-        <v>0</v>
-      </c>
-      <c r="J24" s="12">
+      <c r="L24" s="13">
+        <v>0</v>
+      </c>
+      <c r="M24" s="13">
         <v>1</v>
       </c>
-      <c r="K24" s="12">
+      <c r="N24" s="13">
         <v>9</v>
       </c>
-      <c r="L24" s="12">
+      <c r="O24" s="13">
         <v>50</v>
       </c>
-      <c r="M24" s="12">
+      <c r="P24" s="13">
         <v>250</v>
       </c>
-      <c r="N24" s="12">
+      <c r="Q24" s="13">
         <v>1500</v>
       </c>
-      <c r="O24" s="10">
+      <c r="R24" s="11">
         <v>600</v>
       </c>
-      <c r="P24" s="4"/>
-      <c r="Q24" s="4"/>
-      <c r="R24" s="4"/>
       <c r="S24" s="4"/>
+      <c r="T24" s="4"/>
+      <c r="U24" s="4"/>
+      <c r="V24" s="4"/>
     </row>
-    <row r="25" spans="1:19">
+    <row r="25" spans="1:22">
       <c r="A25" s="8" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B25" s="9">
         <v>300</v>
@@ -2092,46 +2938,58 @@
         <v>16</v>
       </c>
       <c r="E25" s="9">
+        <v>1348</v>
+      </c>
+      <c r="F25" s="9">
+        <f>E25*2</f>
         <v>2696</v>
       </c>
-      <c r="F25" s="9">
+      <c r="G25" s="9">
+        <f t="shared" si="0"/>
+        <v>2696</v>
+      </c>
+      <c r="H25" s="10">
+        <f t="shared" si="1"/>
+        <v>1348</v>
+      </c>
+      <c r="I25" s="9">
         <v>8</v>
       </c>
-      <c r="G25" s="9">
+      <c r="J25" s="9">
         <v>2</v>
       </c>
-      <c r="H25" s="9">
+      <c r="K25" s="9">
         <v>125</v>
       </c>
-      <c r="I25" s="9">
+      <c r="L25" s="9">
         <v>1</v>
       </c>
-      <c r="J25" s="9">
+      <c r="M25" s="9">
         <v>1</v>
       </c>
-      <c r="K25" s="9">
+      <c r="N25" s="9">
         <v>9</v>
       </c>
-      <c r="L25" s="9">
+      <c r="O25" s="9">
         <v>50</v>
       </c>
-      <c r="M25" s="9">
+      <c r="P25" s="9">
         <v>250</v>
       </c>
-      <c r="N25" s="9">
+      <c r="Q25" s="9">
         <v>1800</v>
       </c>
-      <c r="O25" s="11">
+      <c r="R25" s="12">
         <v>400</v>
       </c>
-      <c r="P25" s="4"/>
-      <c r="Q25" s="4"/>
-      <c r="R25" s="4"/>
       <c r="S25" s="4"/>
+      <c r="T25" s="4"/>
+      <c r="U25" s="4"/>
+      <c r="V25" s="4"/>
     </row>
-    <row r="26" spans="1:19">
+    <row r="26" spans="1:22">
       <c r="A26" s="8" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B26" s="9">
         <v>300</v>
@@ -2143,97 +3001,120 @@
         <v>10</v>
       </c>
       <c r="E26" s="9">
+        <v>381</v>
+      </c>
+      <c r="F26" s="9">
+        <f>E26*4</f>
         <v>1524</v>
       </c>
-      <c r="F26" s="9">
+      <c r="G26" s="9">
+        <f t="shared" si="0"/>
+        <v>1524</v>
+      </c>
+      <c r="H26" s="10">
+        <f t="shared" si="1"/>
+        <v>762</v>
+      </c>
+      <c r="I26" s="9">
         <v>8</v>
       </c>
-      <c r="G26" s="9">
+      <c r="J26" s="9">
         <v>2</v>
       </c>
-      <c r="H26" s="9">
+      <c r="K26" s="9">
         <v>60</v>
       </c>
-      <c r="I26" s="9">
+      <c r="L26" s="9">
         <v>1</v>
       </c>
-      <c r="J26" s="9">
+      <c r="M26" s="9">
         <v>1</v>
       </c>
-      <c r="K26" s="9">
+      <c r="N26" s="9">
         <v>9</v>
       </c>
-      <c r="L26" s="9">
+      <c r="O26" s="9">
         <v>50</v>
       </c>
-      <c r="M26" s="9">
+      <c r="P26" s="9">
         <v>250</v>
       </c>
-      <c r="N26" s="9">
+      <c r="Q26" s="9">
         <v>2250</v>
       </c>
-      <c r="O26" s="11">
+      <c r="R26" s="12">
         <v>600</v>
       </c>
-      <c r="P26" s="4"/>
-      <c r="Q26" s="4"/>
-      <c r="R26" s="4"/>
       <c r="S26" s="4"/>
+      <c r="T26" s="4"/>
+      <c r="U26" s="4"/>
+      <c r="V26" s="4"/>
     </row>
-    <row r="27" spans="1:19">
+    <row r="27" spans="1:22">
       <c r="A27" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B27" s="13">
+        <v>300</v>
+      </c>
+      <c r="C27" s="13">
+        <v>9529</v>
+      </c>
+      <c r="D27" s="13">
+        <v>9</v>
+      </c>
+      <c r="E27" s="13">
+        <v>88</v>
+      </c>
+      <c r="F27" s="13">
+        <v>88</v>
+      </c>
+      <c r="G27" s="9">
+        <f t="shared" si="0"/>
+        <v>176</v>
+      </c>
+      <c r="H27" s="10">
+        <f t="shared" si="1"/>
+        <v>440</v>
+      </c>
+      <c r="I27" s="13">
+        <v>5</v>
+      </c>
+      <c r="J27" s="13">
+        <v>0.2</v>
+      </c>
+      <c r="K27" s="13">
+        <v>100</v>
+      </c>
+      <c r="L27" s="13">
+        <v>1</v>
+      </c>
+      <c r="M27" s="13">
+        <v>2</v>
+      </c>
+      <c r="N27" s="13">
+        <v>8</v>
+      </c>
+      <c r="O27" s="13">
         <v>50</v>
       </c>
-      <c r="B27" s="12">
-        <v>300</v>
-      </c>
-      <c r="C27" s="12">
-        <v>9529</v>
-      </c>
-      <c r="D27" s="12">
-        <v>9</v>
-      </c>
-      <c r="E27" s="12">
-        <v>88</v>
-      </c>
-      <c r="F27" s="12">
-        <v>5</v>
-      </c>
-      <c r="G27" s="12">
-        <v>0.2</v>
-      </c>
-      <c r="H27" s="12">
-        <v>100</v>
-      </c>
-      <c r="I27" s="12">
-        <v>1</v>
-      </c>
-      <c r="J27" s="12">
-        <v>2</v>
-      </c>
-      <c r="K27" s="12">
-        <v>8</v>
-      </c>
-      <c r="L27" s="12">
-        <v>50</v>
-      </c>
-      <c r="M27" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="N27" s="12">
+      <c r="P27" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q27" s="13">
         <v>1950</v>
       </c>
-      <c r="O27" s="10">
+      <c r="R27" s="11">
         <v>400</v>
       </c>
-      <c r="P27" s="4"/>
-      <c r="Q27" s="4"/>
-      <c r="R27" s="4"/>
       <c r="S27" s="4"/>
+      <c r="T27" s="4"/>
+      <c r="U27" s="4"/>
+      <c r="V27" s="4"/>
     </row>
-    <row r="28" spans="1:19">
+    <row r="28" spans="1:22">
       <c r="A28" s="8" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B28" s="9">
         <v>400</v>
@@ -2248,94 +3129,116 @@
         <v>75</v>
       </c>
       <c r="F28" s="9">
+        <v>75</v>
+      </c>
+      <c r="G28" s="9">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+      <c r="H28" s="10">
+        <f t="shared" si="1"/>
+        <v>750</v>
+      </c>
+      <c r="I28" s="9">
         <v>15</v>
       </c>
-      <c r="G28" s="9">
+      <c r="J28" s="9">
         <v>0.1</v>
       </c>
-      <c r="H28" s="9">
+      <c r="K28" s="9">
         <v>95</v>
       </c>
-      <c r="I28" s="9">
-        <v>0</v>
-      </c>
-      <c r="J28" s="9">
+      <c r="L28" s="9">
+        <v>0</v>
+      </c>
+      <c r="M28" s="9">
         <v>1</v>
       </c>
-      <c r="K28" s="9">
+      <c r="N28" s="9">
         <v>16</v>
       </c>
-      <c r="L28" s="9">
+      <c r="O28" s="9">
         <v>200</v>
       </c>
-      <c r="M28" s="9">
+      <c r="P28" s="9">
         <v>350</v>
       </c>
-      <c r="N28" s="9">
+      <c r="Q28" s="9">
         <v>2200</v>
       </c>
-      <c r="O28" s="11">
+      <c r="R28" s="12">
         <v>800</v>
       </c>
-      <c r="P28" s="4"/>
-      <c r="Q28" s="4"/>
-      <c r="R28" s="4"/>
       <c r="S28" s="4"/>
+      <c r="T28" s="4"/>
+      <c r="U28" s="4"/>
+      <c r="V28" s="4"/>
     </row>
-    <row r="29" spans="1:19">
+    <row r="29" spans="1:22">
       <c r="A29" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="B29" s="12">
+        <v>56</v>
+      </c>
+      <c r="B29" s="13">
         <v>400</v>
       </c>
-      <c r="C29" s="12">
+      <c r="C29" s="13">
         <v>48645</v>
       </c>
-      <c r="D29" s="12">
+      <c r="D29" s="13">
         <v>16</v>
       </c>
-      <c r="E29" s="12">
+      <c r="E29" s="13">
         <v>9726</v>
       </c>
-      <c r="F29" s="12">
+      <c r="F29" s="13">
+        <v>9726</v>
+      </c>
+      <c r="G29" s="9">
+        <f t="shared" si="0"/>
+        <v>9726</v>
+      </c>
+      <c r="H29" s="10">
+        <f t="shared" si="1"/>
+        <v>3890.4</v>
+      </c>
+      <c r="I29" s="13">
         <v>12</v>
       </c>
-      <c r="G29" s="12">
+      <c r="J29" s="13">
         <v>2.5</v>
       </c>
-      <c r="H29" s="12">
-        <v>0</v>
-      </c>
-      <c r="I29" s="12">
+      <c r="K29" s="13">
+        <v>0</v>
+      </c>
+      <c r="L29" s="13">
         <v>0.5</v>
       </c>
-      <c r="J29" s="12">
+      <c r="M29" s="13">
         <v>1</v>
       </c>
-      <c r="K29" s="12">
+      <c r="N29" s="13">
         <v>16</v>
       </c>
-      <c r="L29" s="12">
+      <c r="O29" s="13">
         <v>200</v>
       </c>
-      <c r="M29" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="N29" s="12">
+      <c r="P29" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q29" s="13">
         <v>2000</v>
       </c>
-      <c r="O29" s="10">
+      <c r="R29" s="11">
         <v>800</v>
       </c>
-      <c r="P29" s="4"/>
-      <c r="Q29" s="4"/>
-      <c r="R29" s="4"/>
       <c r="S29" s="4"/>
+      <c r="T29" s="4"/>
+      <c r="U29" s="4"/>
+      <c r="V29" s="4"/>
     </row>
-    <row r="30" spans="1:19">
+    <row r="30" spans="1:22">
       <c r="A30" s="8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B30" s="9">
         <v>400</v>
@@ -2350,43 +3253,54 @@
         <v>6524</v>
       </c>
       <c r="F30" s="9">
+        <v>6524</v>
+      </c>
+      <c r="G30" s="9">
+        <f t="shared" si="0"/>
+        <v>6524</v>
+      </c>
+      <c r="H30" s="10">
+        <f t="shared" si="1"/>
+        <v>3624.44444444444</v>
+      </c>
+      <c r="I30" s="9">
         <v>5</v>
       </c>
-      <c r="G30" s="9">
+      <c r="J30" s="9">
         <v>1.8</v>
       </c>
-      <c r="H30" s="9">
+      <c r="K30" s="9">
         <v>100</v>
       </c>
-      <c r="I30" s="9">
-        <v>0</v>
-      </c>
-      <c r="J30" s="9">
+      <c r="L30" s="9">
+        <v>0</v>
+      </c>
+      <c r="M30" s="9">
         <v>1</v>
       </c>
-      <c r="K30" s="9">
+      <c r="N30" s="9">
         <v>16</v>
       </c>
-      <c r="L30" s="9">
+      <c r="O30" s="9">
         <v>200</v>
       </c>
-      <c r="M30" s="9">
+      <c r="P30" s="9">
         <v>350</v>
       </c>
-      <c r="N30" s="9">
+      <c r="Q30" s="9">
         <v>1600</v>
       </c>
-      <c r="O30" s="11">
+      <c r="R30" s="12">
         <v>800</v>
       </c>
-      <c r="P30" s="4"/>
-      <c r="Q30" s="4"/>
-      <c r="R30" s="4"/>
       <c r="S30" s="4"/>
+      <c r="T30" s="4"/>
+      <c r="U30" s="4"/>
+      <c r="V30" s="4"/>
     </row>
-    <row r="31" spans="1:19">
+    <row r="31" spans="1:22">
       <c r="A31" s="8" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B31" s="9">
         <v>400</v>
@@ -2401,145 +3315,179 @@
         <v>7952</v>
       </c>
       <c r="F31" s="9">
+        <v>7952</v>
+      </c>
+      <c r="G31" s="9">
+        <f t="shared" si="0"/>
+        <v>7952</v>
+      </c>
+      <c r="H31" s="10">
+        <f t="shared" si="1"/>
+        <v>39760</v>
+      </c>
+      <c r="I31" s="9">
         <v>3</v>
       </c>
-      <c r="G31" s="9">
+      <c r="J31" s="9">
         <v>0.2</v>
       </c>
-      <c r="H31" s="9">
+      <c r="K31" s="9">
         <v>115</v>
       </c>
-      <c r="I31" s="9">
+      <c r="L31" s="9">
         <v>1</v>
       </c>
-      <c r="J31" s="9">
+      <c r="M31" s="9">
         <v>1</v>
       </c>
-      <c r="K31" s="9">
+      <c r="N31" s="9">
         <v>16</v>
       </c>
-      <c r="L31" s="9">
+      <c r="O31" s="9">
         <v>200</v>
       </c>
-      <c r="M31" s="9">
+      <c r="P31" s="9">
         <v>350</v>
       </c>
-      <c r="N31" s="9">
+      <c r="Q31" s="9">
         <v>1400</v>
       </c>
-      <c r="O31" s="11">
+      <c r="R31" s="12">
         <v>800</v>
       </c>
-      <c r="P31" s="4"/>
-      <c r="Q31" s="4"/>
-      <c r="R31" s="4"/>
       <c r="S31" s="4"/>
+      <c r="T31" s="4"/>
+      <c r="U31" s="4"/>
+      <c r="V31" s="4"/>
     </row>
-    <row r="32" spans="1:19">
+    <row r="32" spans="1:22">
       <c r="A32" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="B32" s="12">
+        <v>60</v>
+      </c>
+      <c r="B32" s="13">
         <v>400</v>
       </c>
-      <c r="C32" s="12">
+      <c r="C32" s="13">
         <v>16065</v>
       </c>
-      <c r="D32" s="12">
+      <c r="D32" s="13">
         <v>10</v>
       </c>
-      <c r="E32" s="12">
+      <c r="E32" s="13">
         <v>5027</v>
       </c>
-      <c r="F32" s="12">
-        <v>0</v>
-      </c>
-      <c r="G32" s="12">
-        <v>4.5999999999999996</v>
-      </c>
-      <c r="H32" s="12">
+      <c r="F32" s="13">
+        <v>5027</v>
+      </c>
+      <c r="G32" s="9">
+        <f>F32*M32*3</f>
+        <v>15081</v>
+      </c>
+      <c r="H32" s="10">
+        <f t="shared" si="1"/>
+        <v>1092.82608695652</v>
+      </c>
+      <c r="I32" s="13">
+        <v>0</v>
+      </c>
+      <c r="J32" s="13">
+        <v>4.6</v>
+      </c>
+      <c r="K32" s="13">
         <v>110</v>
       </c>
-      <c r="I32" s="12">
+      <c r="L32" s="13">
         <v>1</v>
       </c>
-      <c r="J32" s="12">
+      <c r="M32" s="13">
         <v>1</v>
       </c>
-      <c r="K32" s="12">
+      <c r="N32" s="13">
         <v>16</v>
       </c>
-      <c r="L32" s="12">
+      <c r="O32" s="13">
         <v>200</v>
       </c>
-      <c r="M32" s="12">
+      <c r="P32" s="13">
         <v>350</v>
       </c>
-      <c r="N32" s="12">
+      <c r="Q32" s="13">
         <v>2400</v>
       </c>
-      <c r="O32" s="10">
+      <c r="R32" s="11">
         <v>800</v>
       </c>
-      <c r="P32" s="4"/>
-      <c r="Q32" s="4"/>
-      <c r="R32" s="4"/>
       <c r="S32" s="4"/>
+      <c r="T32" s="4"/>
+      <c r="U32" s="4"/>
+      <c r="V32" s="4"/>
     </row>
-    <row r="33" spans="1:19">
+    <row r="33" spans="1:22">
       <c r="A33" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="B33" s="12">
+        <v>61</v>
+      </c>
+      <c r="B33" s="13">
         <v>500</v>
       </c>
-      <c r="C33" s="12">
+      <c r="C33" s="13">
         <v>21339</v>
       </c>
-      <c r="D33" s="12">
+      <c r="D33" s="13">
         <v>10</v>
       </c>
-      <c r="E33" s="14">
+      <c r="E33" s="15">
+        <v>4742</v>
+      </c>
+      <c r="F33" s="15">
+        <f>E33*4</f>
         <v>18968</v>
       </c>
-      <c r="F33" s="12">
+      <c r="G33" s="9">
+        <f t="shared" si="0"/>
+        <v>18968</v>
+      </c>
+      <c r="H33" s="10">
+        <f t="shared" si="1"/>
+        <v>4123.47826086957</v>
+      </c>
+      <c r="I33" s="13">
         <v>7</v>
       </c>
-      <c r="G33" s="12">
-        <v>4.5999999999999996</v>
-      </c>
-      <c r="H33" s="12">
+      <c r="J33" s="13">
+        <v>4.6</v>
+      </c>
+      <c r="K33" s="13">
         <v>120</v>
       </c>
-      <c r="I33" s="12">
+      <c r="L33" s="13">
         <v>1</v>
       </c>
-      <c r="J33" s="12">
+      <c r="M33" s="13">
         <v>1</v>
       </c>
-      <c r="K33" s="12">
+      <c r="N33" s="13">
         <v>25</v>
       </c>
-      <c r="L33" s="12">
+      <c r="O33" s="13">
         <v>200</v>
       </c>
-      <c r="M33" s="12">
+      <c r="P33" s="13">
         <v>400</v>
       </c>
-      <c r="N33" s="12">
+      <c r="Q33" s="13">
         <v>1750</v>
       </c>
-      <c r="O33" s="10">
+      <c r="R33" s="11">
         <v>1000</v>
       </c>
-      <c r="P33" s="4"/>
-      <c r="Q33" s="4"/>
-      <c r="R33" s="4"/>
       <c r="S33" s="4"/>
+      <c r="T33" s="4"/>
+      <c r="U33" s="4"/>
+      <c r="V33" s="4"/>
     </row>
-    <row r="34" spans="1:19">
+    <row r="34" spans="1:22">
       <c r="A34" s="8" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B34" s="9">
         <v>800</v>
@@ -2550,47 +3498,58 @@
       <c r="D34" s="9">
         <v>10</v>
       </c>
-      <c r="E34" s="15">
+      <c r="E34" s="16">
         <v>3859</v>
       </c>
-      <c r="F34" s="9">
+      <c r="F34" s="16">
+        <v>3859</v>
+      </c>
+      <c r="G34" s="9">
+        <f>F34*M34*10</f>
+        <v>38590</v>
+      </c>
+      <c r="H34" s="10">
+        <f>G34/J34</f>
+        <v>9647.5</v>
+      </c>
+      <c r="I34" s="9">
         <v>10</v>
       </c>
-      <c r="G34" s="9">
+      <c r="J34" s="9">
         <v>4</v>
       </c>
-      <c r="H34" s="9">
+      <c r="K34" s="9">
         <v>100</v>
       </c>
-      <c r="I34" s="9">
+      <c r="L34" s="9">
         <v>1</v>
       </c>
-      <c r="J34" s="9">
+      <c r="M34" s="9">
         <v>1</v>
       </c>
-      <c r="K34" s="9">
+      <c r="N34" s="9">
         <v>49</v>
       </c>
-      <c r="L34" s="9">
+      <c r="O34" s="9">
         <v>350</v>
       </c>
-      <c r="M34" s="9">
+      <c r="P34" s="9">
         <v>500</v>
       </c>
-      <c r="N34" s="9">
+      <c r="Q34" s="9">
         <v>4800</v>
       </c>
-      <c r="O34" s="11">
+      <c r="R34" s="12">
         <v>1600</v>
       </c>
-      <c r="P34" s="4"/>
-      <c r="Q34" s="4"/>
-      <c r="R34" s="4"/>
       <c r="S34" s="4"/>
+      <c r="T34" s="4"/>
+      <c r="U34" s="4"/>
+      <c r="V34" s="4"/>
     </row>
-    <row r="35" spans="1:19">
+    <row r="35" spans="1:22">
       <c r="A35" s="8" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B35" s="9">
         <v>800</v>
@@ -2601,176 +3560,214 @@
       <c r="D35" s="9">
         <v>6</v>
       </c>
-      <c r="E35" s="15">
+      <c r="E35" s="16">
+        <v>5899</v>
+      </c>
+      <c r="F35" s="16">
+        <f>E35*4</f>
         <v>23596</v>
       </c>
-      <c r="F35" s="9">
+      <c r="G35" s="9">
+        <f t="shared" si="0"/>
+        <v>23596</v>
+      </c>
+      <c r="H35" s="10">
+        <f t="shared" si="1"/>
+        <v>11798</v>
+      </c>
+      <c r="I35" s="9">
         <v>5</v>
       </c>
-      <c r="G35" s="9">
+      <c r="J35" s="9">
         <v>2</v>
       </c>
-      <c r="H35" s="9">
+      <c r="K35" s="9">
         <v>100</v>
       </c>
-      <c r="I35" s="9">
+      <c r="L35" s="9">
         <v>0.5</v>
       </c>
-      <c r="J35" s="9">
+      <c r="M35" s="9">
         <v>1</v>
       </c>
-      <c r="K35" s="9">
+      <c r="N35" s="9">
         <v>49</v>
       </c>
-      <c r="L35" s="9">
+      <c r="O35" s="9">
         <v>350</v>
       </c>
-      <c r="M35" s="9">
+      <c r="P35" s="9">
         <v>500</v>
       </c>
-      <c r="N35" s="9">
+      <c r="Q35" s="9">
         <v>3200</v>
       </c>
-      <c r="O35" s="11">
+      <c r="R35" s="12">
         <v>1600</v>
       </c>
-      <c r="P35" s="4"/>
-      <c r="Q35" s="4"/>
-      <c r="R35" s="4"/>
       <c r="S35" s="4"/>
+      <c r="T35" s="4"/>
+      <c r="U35" s="4"/>
+      <c r="V35" s="4"/>
     </row>
-    <row r="36" spans="1:19">
+    <row r="36" spans="1:22">
       <c r="A36" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="B36" s="12">
+        <v>64</v>
+      </c>
+      <c r="B36" s="13">
         <v>800</v>
       </c>
-      <c r="C36" s="12">
+      <c r="C36" s="13">
         <v>113593</v>
       </c>
-      <c r="D36" s="12">
+      <c r="D36" s="13">
         <v>6</v>
       </c>
-      <c r="E36" s="14">
+      <c r="E36" s="15">
+        <v>7520</v>
+      </c>
+      <c r="F36" s="15">
+        <f>E36*2</f>
         <v>15040</v>
       </c>
-      <c r="F36" s="12">
+      <c r="G36" s="9">
+        <f t="shared" si="0"/>
+        <v>15040</v>
+      </c>
+      <c r="H36" s="10">
+        <f t="shared" si="1"/>
+        <v>8355.55555555555</v>
+      </c>
+      <c r="I36" s="13">
         <v>4.5</v>
       </c>
-      <c r="G36" s="12">
+      <c r="J36" s="13">
         <v>1.8</v>
       </c>
-      <c r="H36" s="12">
+      <c r="K36" s="13">
         <v>100</v>
       </c>
-      <c r="I36" s="12">
-        <v>0</v>
-      </c>
-      <c r="J36" s="12">
+      <c r="L36" s="13">
+        <v>0</v>
+      </c>
+      <c r="M36" s="13">
         <v>1</v>
       </c>
-      <c r="K36" s="12">
+      <c r="N36" s="13">
         <v>49</v>
       </c>
-      <c r="L36" s="12">
+      <c r="O36" s="13">
         <v>350</v>
       </c>
-      <c r="M36" s="12">
+      <c r="P36" s="13">
         <v>500</v>
       </c>
-      <c r="N36" s="12">
+      <c r="Q36" s="13">
         <v>3200</v>
       </c>
-      <c r="O36" s="10">
+      <c r="R36" s="11">
         <v>1600</v>
       </c>
-      <c r="P36" s="4"/>
-      <c r="Q36" s="4"/>
-      <c r="R36" s="4"/>
       <c r="S36" s="4"/>
+      <c r="T36" s="4"/>
+      <c r="U36" s="4"/>
+      <c r="V36" s="4"/>
     </row>
-    <row r="37" spans="1:19">
+    <row r="37" spans="1:22">
       <c r="A37" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="B37" s="12">
+        <v>65</v>
+      </c>
+      <c r="B37" s="13">
         <v>800</v>
       </c>
-      <c r="C37" s="12">
+      <c r="C37" s="13">
         <v>125512</v>
       </c>
-      <c r="D37" s="12">
+      <c r="D37" s="13">
         <v>6</v>
       </c>
-      <c r="E37" s="14">
+      <c r="E37" s="15">
         <v>9798</v>
       </c>
-      <c r="F37" s="12">
+      <c r="F37" s="15">
+        <v>9798</v>
+      </c>
+      <c r="G37" s="9">
+        <f t="shared" si="0"/>
+        <v>9798</v>
+      </c>
+      <c r="H37" s="10">
+        <f t="shared" si="1"/>
+        <v>48990</v>
+      </c>
+      <c r="I37" s="13">
         <v>3</v>
       </c>
-      <c r="G37" s="12">
+      <c r="J37" s="13">
         <v>0.2</v>
       </c>
-      <c r="H37" s="12">
+      <c r="K37" s="13">
         <v>115</v>
       </c>
-      <c r="I37" s="12">
+      <c r="L37" s="13">
         <v>1</v>
       </c>
-      <c r="J37" s="12">
+      <c r="M37" s="13">
         <v>1</v>
       </c>
-      <c r="K37" s="12">
+      <c r="N37" s="13">
         <v>49</v>
       </c>
-      <c r="L37" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="M37" s="12">
+      <c r="O37" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="P37" s="13">
         <v>500</v>
       </c>
-      <c r="N37" s="12">
+      <c r="Q37" s="13">
         <v>3200</v>
       </c>
-      <c r="O37" s="10">
+      <c r="R37" s="11">
         <v>1600</v>
       </c>
-      <c r="P37" s="4"/>
-      <c r="Q37" s="4"/>
-      <c r="R37" s="4"/>
       <c r="S37" s="4"/>
+      <c r="T37" s="4"/>
+      <c r="U37" s="4"/>
+      <c r="V37" s="4"/>
     </row>
-    <row r="38" spans="1:19" ht="14.6">
-      <c r="A38" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="B38" s="17"/>
-      <c r="C38" s="17"/>
-      <c r="D38" s="17" t="s">
-        <v>65</v>
-      </c>
-      <c r="E38" s="17"/>
-      <c r="F38" s="17"/>
-      <c r="G38" s="17"/>
-      <c r="H38" s="17"/>
-      <c r="I38" s="17"/>
-      <c r="J38" s="17"/>
-      <c r="K38" s="17"/>
-      <c r="L38" s="17"/>
-      <c r="M38" s="17"/>
-      <c r="N38" s="17"/>
-      <c r="O38" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="P38" s="4"/>
-      <c r="Q38" s="4"/>
-      <c r="R38" s="4"/>
+    <row r="38" ht="14.55" spans="1:22">
+      <c r="A38" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="B38" s="18"/>
+      <c r="C38" s="18"/>
+      <c r="D38" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="E38" s="18"/>
+      <c r="F38" s="18"/>
+      <c r="G38" s="18"/>
+      <c r="H38" s="19"/>
+      <c r="I38" s="18"/>
+      <c r="J38" s="18"/>
+      <c r="K38" s="18"/>
+      <c r="L38" s="18"/>
+      <c r="M38" s="18"/>
+      <c r="N38" s="18"/>
+      <c r="O38" s="18"/>
+      <c r="P38" s="18"/>
+      <c r="Q38" s="18"/>
+      <c r="R38" s="18" t="s">
+        <v>69</v>
+      </c>
       <c r="S38" s="4"/>
+      <c r="T38" s="4"/>
+      <c r="U38" s="4"/>
+      <c r="V38" s="4"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>